<commit_message>
cambios en mapa y semaforo cutaneo
</commit_message>
<xml_diff>
--- a/FERMONT.xlsx
+++ b/FERMONT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\QRSIS05\Desktop\fermont\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21E6051C-3FE2-4A0D-B8A8-5A0B256EBD01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6151E1A3-A00D-40E6-A33B-C9114896B403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4CEBE4EC-E555-4787-B0CC-888459687361}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="206">
   <si>
     <t>PASO 1</t>
   </si>
@@ -588,6 +588,75 @@
   </si>
   <si>
     <t>DESPUÉS DE ÁCNE</t>
+  </si>
+  <si>
+    <t>PASO 11</t>
+  </si>
+  <si>
+    <t>PREGUNTAS CORPORALES</t>
+  </si>
+  <si>
+    <t>Circulación</t>
+  </si>
+  <si>
+    <t>¿Tienes piernas cansadas?</t>
+  </si>
+  <si>
+    <t>¿Varices?</t>
+  </si>
+  <si>
+    <t>¿Retención de líquidos?</t>
+  </si>
+  <si>
+    <t>¿Dolor al tacto?</t>
+  </si>
+  <si>
+    <t>Peso y hábitos</t>
+  </si>
+  <si>
+    <t>¿Has subido o bajado de peso recientemente?</t>
+  </si>
+  <si>
+    <t>¿Tu peso fluctúa mucho?</t>
+  </si>
+  <si>
+    <t>Actividad física</t>
+  </si>
+  <si>
+    <t>¿Haces ejercicio?</t>
+  </si>
+  <si>
+    <t>Objetivos</t>
+  </si>
+  <si>
+    <t>¿Qué zona deseas mejorar más?</t>
+  </si>
+  <si>
+    <t>¿Qué es lo que más te incomoda visualmente?</t>
+  </si>
+  <si>
+    <t>VALORACIONES</t>
+  </si>
+  <si>
+    <t>11 PASOS DE VALORACION O MENOS SI ES CLIENTE RECURRENTE</t>
+  </si>
+  <si>
+    <t>MAPA INTERACTIVO</t>
+  </si>
+  <si>
+    <t>FOTOGRAFIAS CLINICAS</t>
+  </si>
+  <si>
+    <t>SEMÁFORO CUTÁNEO</t>
+  </si>
+  <si>
+    <t>🟢 Verde Piel estable y apta para procedimientos.</t>
+  </si>
+  <si>
+    <t>🟡 Amarillo Piel sensible o sensibilizada.</t>
+  </si>
+  <si>
+    <t>🔴 Rojo Piel contraindicada para procedimientos agresivos.</t>
   </si>
 </sst>
 </file>
@@ -617,7 +686,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -640,11 +709,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -654,13 +736,20 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -995,16 +1084,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D1FF3BB-27F8-41B1-B991-559CB6C2CDE7}">
-  <dimension ref="A1:E150"/>
+  <dimension ref="A1:I160"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="38.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="59.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="44.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="57.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
@@ -1020,12 +1111,18 @@
       <c r="E1" s="1" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="H1" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="I1" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="5" t="s">
         <v>1</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -1033,55 +1130,81 @@
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
+      <c r="H2" s="6"/>
+      <c r="I2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
       <c r="C3" s="3" t="s">
         <v>3</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
+      <c r="H3" s="6"/>
+      <c r="I3" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
       <c r="C4" s="3" t="s">
         <v>4</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
+      <c r="H4" s="6"/>
+      <c r="I4" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="5"/>
+      <c r="B5" s="5"/>
       <c r="C5" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
+      <c r="H5" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="I5" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="5"/>
+      <c r="B6" s="5"/>
       <c r="C6" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="10" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="5"/>
+      <c r="B7" s="5"/>
       <c r="C7" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
+      <c r="H7" s="6"/>
+      <c r="I7" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
       <c r="C8" s="4" t="s">
         <v>8</v>
       </c>
@@ -1090,235 +1213,235 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
       <c r="C9" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="5"/>
+      <c r="B10" s="5"/>
       <c r="C10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="5"/>
+      <c r="B11" s="5"/>
       <c r="C11" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="5"/>
+      <c r="B12" s="5"/>
       <c r="C12" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E13" s="3"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
       <c r="C14" s="5"/>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="3" t="s">
         <v>21</v>
       </c>
       <c r="E14" s="3"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="5"/>
+      <c r="B15" s="5"/>
       <c r="C15" s="5"/>
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="3" t="s">
         <v>22</v>
       </c>
       <c r="E15" s="3"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="5"/>
+      <c r="B16" s="5"/>
       <c r="C16" s="5"/>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="3" t="s">
         <v>23</v>
       </c>
       <c r="E16" s="3"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
       <c r="C17" s="5"/>
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="3" t="s">
         <v>24</v>
       </c>
       <c r="E17" s="3"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
       <c r="C18" s="5"/>
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="3" t="s">
         <v>25</v>
       </c>
       <c r="E18" s="3"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
       <c r="C19" s="5"/>
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="3" t="s">
         <v>26</v>
       </c>
       <c r="E19" s="3"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
       <c r="C20" s="5"/>
-      <c r="D20" s="6" t="s">
+      <c r="D20" s="3" t="s">
         <v>27</v>
       </c>
       <c r="E20" s="3"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
       <c r="C21" s="5"/>
-      <c r="D21" s="6" t="s">
+      <c r="D21" s="3" t="s">
         <v>28</v>
       </c>
       <c r="E21" s="3"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
       <c r="C22" s="5"/>
-      <c r="D22" s="6" t="s">
+      <c r="D22" s="3" t="s">
         <v>29</v>
       </c>
       <c r="E22" s="3"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
       <c r="C23" s="5"/>
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="3" t="s">
         <v>30</v>
       </c>
       <c r="E23" s="3"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
       <c r="C24" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="D24" s="3" t="s">
         <v>32</v>
       </c>
       <c r="E24" s="3"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
+      <c r="A25" s="5"/>
+      <c r="B25" s="5"/>
       <c r="C25" s="5"/>
-      <c r="D25" s="6" t="s">
+      <c r="D25" s="3" t="s">
         <v>33</v>
       </c>
       <c r="E25" s="3"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
+      <c r="A26" s="5"/>
+      <c r="B26" s="5"/>
       <c r="C26" s="5"/>
-      <c r="D26" s="6" t="s">
+      <c r="D26" s="3" t="s">
         <v>29</v>
       </c>
       <c r="E26" s="3"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
+      <c r="A27" s="5"/>
+      <c r="B27" s="5"/>
       <c r="C27" s="5"/>
-      <c r="D27" s="6" t="s">
+      <c r="D27" s="3" t="s">
         <v>34</v>
       </c>
       <c r="E27" s="3"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
+      <c r="A28" s="5"/>
+      <c r="B28" s="5"/>
       <c r="C28" s="5"/>
-      <c r="D28" s="6" t="s">
+      <c r="D28" s="3" t="s">
         <v>35</v>
       </c>
       <c r="E28" s="3"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
+      <c r="A29" s="5"/>
+      <c r="B29" s="5"/>
       <c r="C29" s="5"/>
-      <c r="D29" s="6" t="s">
+      <c r="D29" s="3" t="s">
         <v>36</v>
       </c>
       <c r="E29" s="3"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="2"/>
-      <c r="B30" s="2"/>
+      <c r="A30" s="5"/>
+      <c r="B30" s="5"/>
       <c r="C30" s="5"/>
-      <c r="D30" s="6" t="s">
+      <c r="D30" s="3" t="s">
         <v>37</v>
       </c>
       <c r="E30" s="3"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
+      <c r="A31" s="5"/>
+      <c r="B31" s="5"/>
       <c r="C31" s="5"/>
-      <c r="D31" s="6" t="s">
+      <c r="D31" s="3" t="s">
         <v>38</v>
       </c>
       <c r="E31" s="3"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="2"/>
-      <c r="B32" s="2"/>
+      <c r="A32" s="5"/>
+      <c r="B32" s="5"/>
       <c r="C32" s="5"/>
-      <c r="D32" s="6" t="s">
+      <c r="D32" s="3" t="s">
         <v>28</v>
       </c>
       <c r="E32" s="3"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="2" t="s">
+      <c r="A33" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="5" t="s">
         <v>40</v>
       </c>
       <c r="C33" s="3" t="s">
@@ -1328,8 +1451,8 @@
       <c r="E33" s="3"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2"/>
+      <c r="A34" s="5"/>
+      <c r="B34" s="5"/>
       <c r="C34" s="3" t="s">
         <v>42</v>
       </c>
@@ -1337,8 +1460,8 @@
       <c r="E34" s="3"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="2"/>
-      <c r="B35" s="2"/>
+      <c r="A35" s="5"/>
+      <c r="B35" s="5"/>
       <c r="C35" s="3" t="s">
         <v>43</v>
       </c>
@@ -1346,8 +1469,8 @@
       <c r="E35" s="3"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="2"/>
-      <c r="B36" s="2"/>
+      <c r="A36" s="5"/>
+      <c r="B36" s="5"/>
       <c r="C36" s="3" t="s">
         <v>44</v>
       </c>
@@ -1355,8 +1478,8 @@
       <c r="E36" s="3"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="2"/>
-      <c r="B37" s="2"/>
+      <c r="A37" s="5"/>
+      <c r="B37" s="5"/>
       <c r="C37" s="3" t="s">
         <v>45</v>
       </c>
@@ -1364,13 +1487,13 @@
       <c r="E37" s="3"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="2" t="s">
+      <c r="A38" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="C38" s="5" t="s">
         <v>48</v>
       </c>
       <c r="D38" s="3" t="s">
@@ -1379,108 +1502,108 @@
       <c r="E38" s="3"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="2"/>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
+      <c r="A39" s="5"/>
+      <c r="B39" s="5"/>
+      <c r="C39" s="5"/>
       <c r="D39" s="3" t="s">
         <v>50</v>
       </c>
       <c r="E39" s="3"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="2"/>
-      <c r="B40" s="2"/>
-      <c r="C40" s="2"/>
+      <c r="A40" s="5"/>
+      <c r="B40" s="5"/>
+      <c r="C40" s="5"/>
       <c r="D40" s="3" t="s">
         <v>51</v>
       </c>
       <c r="E40" s="3"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="2"/>
-      <c r="B41" s="2"/>
-      <c r="C41" s="2"/>
+      <c r="A41" s="5"/>
+      <c r="B41" s="5"/>
+      <c r="C41" s="5"/>
       <c r="D41" s="3" t="s">
         <v>52</v>
       </c>
       <c r="E41" s="3"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="2"/>
-      <c r="B42" s="2"/>
-      <c r="C42" s="2"/>
+      <c r="A42" s="5"/>
+      <c r="B42" s="5"/>
+      <c r="C42" s="5"/>
       <c r="D42" s="3" t="s">
         <v>53</v>
       </c>
       <c r="E42" s="3"/>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="2"/>
-      <c r="B43" s="2"/>
-      <c r="C43" s="2"/>
+      <c r="A43" s="5"/>
+      <c r="B43" s="5"/>
+      <c r="C43" s="5"/>
       <c r="D43" s="3" t="s">
         <v>54</v>
       </c>
       <c r="E43" s="3"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="2"/>
-      <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
+      <c r="A44" s="5"/>
+      <c r="B44" s="5"/>
+      <c r="C44" s="5"/>
       <c r="D44" s="3" t="s">
         <v>55</v>
       </c>
       <c r="E44" s="3"/>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" s="2"/>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
+      <c r="A45" s="5"/>
+      <c r="B45" s="5"/>
+      <c r="C45" s="5"/>
       <c r="D45" s="3" t="s">
         <v>56</v>
       </c>
       <c r="E45" s="3"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="2"/>
-      <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
+      <c r="A46" s="5"/>
+      <c r="B46" s="5"/>
+      <c r="C46" s="5"/>
       <c r="D46" s="3" t="s">
         <v>57</v>
       </c>
       <c r="E46" s="3"/>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
+      <c r="A47" s="5"/>
+      <c r="B47" s="5"/>
+      <c r="C47" s="5"/>
       <c r="D47" s="3" t="s">
         <v>58</v>
       </c>
       <c r="E47" s="3"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="2"/>
-      <c r="B48" s="2"/>
-      <c r="C48" s="2"/>
+      <c r="A48" s="5"/>
+      <c r="B48" s="5"/>
+      <c r="C48" s="5"/>
       <c r="D48" s="3" t="s">
         <v>59</v>
       </c>
       <c r="E48" s="3"/>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" s="2"/>
-      <c r="B49" s="2"/>
-      <c r="C49" s="2"/>
+      <c r="A49" s="5"/>
+      <c r="B49" s="5"/>
+      <c r="C49" s="5"/>
       <c r="D49" s="3" t="s">
         <v>86</v>
       </c>
       <c r="E49" s="3"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="2"/>
-      <c r="B50" s="2"/>
-      <c r="C50" s="2" t="s">
+      <c r="A50" s="5"/>
+      <c r="B50" s="5"/>
+      <c r="C50" s="5" t="s">
         <v>61</v>
       </c>
       <c r="D50" s="3" t="s">
@@ -1489,27 +1612,27 @@
       <c r="E50" s="3"/>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="2"/>
-      <c r="B51" s="2"/>
-      <c r="C51" s="2"/>
+      <c r="A51" s="5"/>
+      <c r="B51" s="5"/>
+      <c r="C51" s="5"/>
       <c r="D51" s="3" t="s">
         <v>63</v>
       </c>
       <c r="E51" s="3"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="2"/>
-      <c r="B52" s="2"/>
-      <c r="C52" s="2"/>
+      <c r="A52" s="5"/>
+      <c r="B52" s="5"/>
+      <c r="C52" s="5"/>
       <c r="D52" s="3" t="s">
         <v>64</v>
       </c>
       <c r="E52" s="3"/>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="2"/>
-      <c r="B53" s="2"/>
-      <c r="C53" s="2" t="s">
+      <c r="A53" s="5"/>
+      <c r="B53" s="5"/>
+      <c r="C53" s="5" t="s">
         <v>65</v>
       </c>
       <c r="D53" s="3" t="s">
@@ -1518,63 +1641,63 @@
       <c r="E53" s="3"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="2"/>
-      <c r="B54" s="2"/>
-      <c r="C54" s="2"/>
+      <c r="A54" s="5"/>
+      <c r="B54" s="5"/>
+      <c r="C54" s="5"/>
       <c r="D54" s="3" t="s">
         <v>67</v>
       </c>
       <c r="E54" s="3"/>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" s="2"/>
-      <c r="B55" s="2"/>
-      <c r="C55" s="2"/>
+      <c r="A55" s="5"/>
+      <c r="B55" s="5"/>
+      <c r="C55" s="5"/>
       <c r="D55" s="3" t="s">
         <v>68</v>
       </c>
       <c r="E55" s="3"/>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" s="2"/>
-      <c r="B56" s="2"/>
-      <c r="C56" s="2"/>
+      <c r="A56" s="5"/>
+      <c r="B56" s="5"/>
+      <c r="C56" s="5"/>
       <c r="D56" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E56" s="3"/>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="2"/>
-      <c r="B57" s="2"/>
-      <c r="C57" s="2"/>
+      <c r="A57" s="5"/>
+      <c r="B57" s="5"/>
+      <c r="C57" s="5"/>
       <c r="D57" s="3" t="s">
         <v>70</v>
       </c>
       <c r="E57" s="3"/>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" s="2"/>
-      <c r="B58" s="2"/>
-      <c r="C58" s="2"/>
+      <c r="A58" s="5"/>
+      <c r="B58" s="5"/>
+      <c r="C58" s="5"/>
       <c r="D58" s="3" t="s">
         <v>71</v>
       </c>
       <c r="E58" s="3"/>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" s="2"/>
-      <c r="B59" s="2"/>
-      <c r="C59" s="2"/>
+      <c r="A59" s="5"/>
+      <c r="B59" s="5"/>
+      <c r="C59" s="5"/>
       <c r="D59" s="3" t="s">
         <v>72</v>
       </c>
       <c r="E59" s="3"/>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" s="2"/>
-      <c r="B60" s="2"/>
-      <c r="C60" s="2" t="s">
+      <c r="A60" s="5"/>
+      <c r="B60" s="5"/>
+      <c r="C60" s="5" t="s">
         <v>73</v>
       </c>
       <c r="D60" s="3" t="s">
@@ -1583,109 +1706,109 @@
       <c r="E60" s="3"/>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" s="2"/>
-      <c r="B61" s="2"/>
-      <c r="C61" s="2"/>
+      <c r="A61" s="5"/>
+      <c r="B61" s="5"/>
+      <c r="C61" s="5"/>
       <c r="D61" s="3" t="s">
         <v>75</v>
       </c>
       <c r="E61" s="3"/>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" s="2"/>
-      <c r="B62" s="2"/>
-      <c r="C62" s="2"/>
+      <c r="A62" s="5"/>
+      <c r="B62" s="5"/>
+      <c r="C62" s="5"/>
       <c r="D62" s="3" t="s">
         <v>76</v>
       </c>
       <c r="E62" s="3"/>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" s="2"/>
-      <c r="B63" s="2"/>
-      <c r="C63" s="2"/>
+      <c r="A63" s="5"/>
+      <c r="B63" s="5"/>
+      <c r="C63" s="5"/>
       <c r="D63" s="3" t="s">
         <v>77</v>
       </c>
       <c r="E63" s="3"/>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" s="2"/>
-      <c r="B64" s="2"/>
-      <c r="C64" s="2"/>
+      <c r="A64" s="5"/>
+      <c r="B64" s="5"/>
+      <c r="C64" s="5"/>
       <c r="D64" s="3" t="s">
         <v>78</v>
       </c>
       <c r="E64" s="3"/>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A65" s="2"/>
-      <c r="B65" s="2"/>
-      <c r="C65" s="2"/>
+      <c r="A65" s="5"/>
+      <c r="B65" s="5"/>
+      <c r="C65" s="5"/>
       <c r="D65" s="3" t="s">
         <v>79</v>
       </c>
       <c r="E65" s="3"/>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" s="2"/>
-      <c r="B66" s="2"/>
-      <c r="C66" s="2"/>
+      <c r="A66" s="5"/>
+      <c r="B66" s="5"/>
+      <c r="C66" s="5"/>
       <c r="D66" s="3" t="s">
         <v>80</v>
       </c>
       <c r="E66" s="3"/>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" s="2"/>
-      <c r="B67" s="2"/>
-      <c r="C67" s="2"/>
+      <c r="A67" s="5"/>
+      <c r="B67" s="5"/>
+      <c r="C67" s="5"/>
       <c r="D67" s="3" t="s">
         <v>81</v>
       </c>
       <c r="E67" s="3"/>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" s="2"/>
-      <c r="B68" s="2"/>
-      <c r="C68" s="2"/>
+      <c r="A68" s="5"/>
+      <c r="B68" s="5"/>
+      <c r="C68" s="5"/>
       <c r="D68" s="3" t="s">
         <v>82</v>
       </c>
       <c r="E68" s="3"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="2"/>
-      <c r="B69" s="2"/>
-      <c r="C69" s="2"/>
+      <c r="A69" s="5"/>
+      <c r="B69" s="5"/>
+      <c r="C69" s="5"/>
       <c r="D69" s="3" t="s">
         <v>83</v>
       </c>
       <c r="E69" s="3"/>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="2"/>
-      <c r="B70" s="2"/>
-      <c r="C70" s="2"/>
+      <c r="A70" s="5"/>
+      <c r="B70" s="5"/>
+      <c r="C70" s="5"/>
       <c r="D70" s="3" t="s">
         <v>84</v>
       </c>
       <c r="E70" s="3"/>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" s="2"/>
-      <c r="B71" s="2"/>
-      <c r="C71" s="2"/>
+      <c r="A71" s="5"/>
+      <c r="B71" s="5"/>
+      <c r="C71" s="5"/>
       <c r="D71" s="3" t="s">
         <v>85</v>
       </c>
       <c r="E71" s="3"/>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" s="2" t="s">
+      <c r="A72" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B72" s="2" t="s">
+      <c r="B72" s="5" t="s">
         <v>88</v>
       </c>
       <c r="C72" s="3" t="s">
@@ -1695,8 +1818,8 @@
       <c r="E72" s="3"/>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A73" s="2"/>
-      <c r="B73" s="2"/>
+      <c r="A73" s="5"/>
+      <c r="B73" s="5"/>
       <c r="C73" s="3" t="s">
         <v>90</v>
       </c>
@@ -1704,8 +1827,8 @@
       <c r="E73" s="3"/>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A74" s="2"/>
-      <c r="B74" s="2"/>
+      <c r="A74" s="5"/>
+      <c r="B74" s="5"/>
       <c r="C74" s="3" t="s">
         <v>91</v>
       </c>
@@ -1713,8 +1836,8 @@
       <c r="E74" s="3"/>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A75" s="2"/>
-      <c r="B75" s="2"/>
+      <c r="A75" s="5"/>
+      <c r="B75" s="5"/>
       <c r="C75" s="3" t="s">
         <v>92</v>
       </c>
@@ -1722,8 +1845,8 @@
       <c r="E75" s="3"/>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A76" s="2"/>
-      <c r="B76" s="2"/>
+      <c r="A76" s="5"/>
+      <c r="B76" s="5"/>
       <c r="C76" s="3" t="s">
         <v>93</v>
       </c>
@@ -1731,8 +1854,8 @@
       <c r="E76" s="3"/>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A77" s="2"/>
-      <c r="B77" s="2"/>
+      <c r="A77" s="5"/>
+      <c r="B77" s="5"/>
       <c r="C77" s="3" t="s">
         <v>94</v>
       </c>
@@ -1740,8 +1863,8 @@
       <c r="E77" s="3"/>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A78" s="2"/>
-      <c r="B78" s="2"/>
+      <c r="A78" s="5"/>
+      <c r="B78" s="5"/>
       <c r="C78" s="3" t="s">
         <v>95</v>
       </c>
@@ -1749,8 +1872,8 @@
       <c r="E78" s="3"/>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A79" s="2"/>
-      <c r="B79" s="2"/>
+      <c r="A79" s="5"/>
+      <c r="B79" s="5"/>
       <c r="C79" s="3" t="s">
         <v>96</v>
       </c>
@@ -1758,8 +1881,8 @@
       <c r="E79" s="3"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A80" s="2"/>
-      <c r="B80" s="2"/>
+      <c r="A80" s="5"/>
+      <c r="B80" s="5"/>
       <c r="C80" s="3" t="s">
         <v>97</v>
       </c>
@@ -1767,8 +1890,8 @@
       <c r="E80" s="3"/>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A81" s="2"/>
-      <c r="B81" s="2"/>
+      <c r="A81" s="5"/>
+      <c r="B81" s="5"/>
       <c r="C81" s="3" t="s">
         <v>98</v>
       </c>
@@ -1776,10 +1899,10 @@
       <c r="E81" s="3"/>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A82" s="2" t="s">
+      <c r="A82" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B82" s="2" t="s">
+      <c r="B82" s="5" t="s">
         <v>100</v>
       </c>
       <c r="C82" s="3" t="s">
@@ -1789,8 +1912,8 @@
       <c r="E82" s="3"/>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A83" s="2"/>
-      <c r="B83" s="2"/>
+      <c r="A83" s="5"/>
+      <c r="B83" s="5"/>
       <c r="C83" s="3" t="s">
         <v>102</v>
       </c>
@@ -1798,8 +1921,8 @@
       <c r="E83" s="3"/>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A84" s="2"/>
-      <c r="B84" s="2"/>
+      <c r="A84" s="5"/>
+      <c r="B84" s="5"/>
       <c r="C84" s="3" t="s">
         <v>103</v>
       </c>
@@ -1807,8 +1930,8 @@
       <c r="E84" s="3"/>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A85" s="2"/>
-      <c r="B85" s="2"/>
+      <c r="A85" s="5"/>
+      <c r="B85" s="5"/>
       <c r="C85" s="3" t="s">
         <v>104</v>
       </c>
@@ -1816,8 +1939,8 @@
       <c r="E85" s="3"/>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A86" s="2"/>
-      <c r="B86" s="2"/>
+      <c r="A86" s="5"/>
+      <c r="B86" s="5"/>
       <c r="C86" s="3" t="s">
         <v>105</v>
       </c>
@@ -1825,13 +1948,13 @@
       <c r="E86" s="3"/>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A87" s="2" t="s">
+      <c r="A87" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="B87" s="2" t="s">
+      <c r="B87" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="C87" s="2" t="s">
+      <c r="C87" s="5" t="s">
         <v>108</v>
       </c>
       <c r="D87" s="3" t="s">
@@ -1840,45 +1963,45 @@
       <c r="E87" s="3"/>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A88" s="2"/>
-      <c r="B88" s="2"/>
-      <c r="C88" s="2"/>
+      <c r="A88" s="5"/>
+      <c r="B88" s="5"/>
+      <c r="C88" s="5"/>
       <c r="D88" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E88" s="3"/>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A89" s="2"/>
-      <c r="B89" s="2"/>
-      <c r="C89" s="2"/>
+      <c r="A89" s="5"/>
+      <c r="B89" s="5"/>
+      <c r="C89" s="5"/>
       <c r="D89" s="3" t="s">
         <v>111</v>
       </c>
       <c r="E89" s="3"/>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A90" s="2"/>
-      <c r="B90" s="2"/>
-      <c r="C90" s="2"/>
+      <c r="A90" s="5"/>
+      <c r="B90" s="5"/>
+      <c r="C90" s="5"/>
       <c r="D90" s="3" t="s">
         <v>112</v>
       </c>
       <c r="E90" s="3"/>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A91" s="2"/>
-      <c r="B91" s="2"/>
-      <c r="C91" s="2"/>
+      <c r="A91" s="5"/>
+      <c r="B91" s="5"/>
+      <c r="C91" s="5"/>
       <c r="D91" s="3" t="s">
         <v>113</v>
       </c>
       <c r="E91" s="3"/>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A92" s="2"/>
-      <c r="B92" s="2"/>
-      <c r="C92" s="7" t="s">
+      <c r="A92" s="5"/>
+      <c r="B92" s="5"/>
+      <c r="C92" s="2" t="s">
         <v>114</v>
       </c>
       <c r="D92" s="3" t="s">
@@ -1887,8 +2010,8 @@
       <c r="E92" s="3"/>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A93" s="2"/>
-      <c r="B93" s="2"/>
+      <c r="A93" s="5"/>
+      <c r="B93" s="5"/>
       <c r="C93" s="1" t="s">
         <v>115</v>
       </c>
@@ -1898,9 +2021,9 @@
       <c r="E93" s="3"/>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A94" s="2"/>
-      <c r="B94" s="2"/>
-      <c r="C94" s="2" t="s">
+      <c r="A94" s="5"/>
+      <c r="B94" s="5"/>
+      <c r="C94" s="5" t="s">
         <v>116</v>
       </c>
       <c r="D94" s="3" t="s">
@@ -1909,49 +2032,49 @@
       <c r="E94" s="3"/>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A95" s="2"/>
-      <c r="B95" s="2"/>
-      <c r="C95" s="2"/>
+      <c r="A95" s="5"/>
+      <c r="B95" s="5"/>
+      <c r="C95" s="5"/>
       <c r="D95" s="3" t="s">
         <v>118</v>
       </c>
       <c r="E95" s="3"/>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A96" s="2"/>
-      <c r="B96" s="2"/>
-      <c r="C96" s="2"/>
+      <c r="A96" s="5"/>
+      <c r="B96" s="5"/>
+      <c r="C96" s="5"/>
       <c r="D96" s="3" t="s">
         <v>119</v>
       </c>
       <c r="E96" s="3"/>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A97" s="2"/>
-      <c r="B97" s="2"/>
-      <c r="C97" s="2"/>
+      <c r="A97" s="5"/>
+      <c r="B97" s="5"/>
+      <c r="C97" s="5"/>
       <c r="D97" s="3" t="s">
         <v>120</v>
       </c>
       <c r="E97" s="3"/>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A98" s="2"/>
-      <c r="B98" s="2"/>
-      <c r="C98" s="2"/>
+      <c r="A98" s="5"/>
+      <c r="B98" s="5"/>
+      <c r="C98" s="5"/>
       <c r="D98" s="3" t="s">
         <v>121</v>
       </c>
       <c r="E98" s="3"/>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A99" s="2" t="s">
+      <c r="A99" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="B99" s="2" t="s">
+      <c r="B99" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="C99" s="2" t="s">
+      <c r="C99" s="5" t="s">
         <v>125</v>
       </c>
       <c r="D99" s="3" t="s">
@@ -1960,45 +2083,45 @@
       <c r="E99" s="3"/>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A100" s="2"/>
-      <c r="B100" s="2"/>
-      <c r="C100" s="2"/>
+      <c r="A100" s="5"/>
+      <c r="B100" s="5"/>
+      <c r="C100" s="5"/>
       <c r="D100" s="3" t="s">
         <v>127</v>
       </c>
       <c r="E100" s="3"/>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A101" s="2"/>
-      <c r="B101" s="2"/>
-      <c r="C101" s="2"/>
+      <c r="A101" s="5"/>
+      <c r="B101" s="5"/>
+      <c r="C101" s="5"/>
       <c r="D101" s="3" t="s">
         <v>128</v>
       </c>
       <c r="E101" s="3"/>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A102" s="2"/>
-      <c r="B102" s="2"/>
-      <c r="C102" s="2"/>
+      <c r="A102" s="5"/>
+      <c r="B102" s="5"/>
+      <c r="C102" s="5"/>
       <c r="D102" s="3" t="s">
         <v>129</v>
       </c>
       <c r="E102" s="3"/>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A103" s="2"/>
-      <c r="B103" s="2"/>
-      <c r="C103" s="2"/>
+      <c r="A103" s="5"/>
+      <c r="B103" s="5"/>
+      <c r="C103" s="5"/>
       <c r="D103" s="3" t="s">
         <v>130</v>
       </c>
       <c r="E103" s="3"/>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A104" s="2"/>
-      <c r="B104" s="2"/>
-      <c r="C104" s="2" t="s">
+      <c r="A104" s="5"/>
+      <c r="B104" s="5"/>
+      <c r="C104" s="5" t="s">
         <v>131</v>
       </c>
       <c r="D104" s="3" t="s">
@@ -2007,45 +2130,45 @@
       <c r="E104" s="3"/>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A105" s="2"/>
-      <c r="B105" s="2"/>
-      <c r="C105" s="2"/>
+      <c r="A105" s="5"/>
+      <c r="B105" s="5"/>
+      <c r="C105" s="5"/>
       <c r="D105" s="3" t="s">
         <v>133</v>
       </c>
       <c r="E105" s="3"/>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A106" s="2"/>
-      <c r="B106" s="2"/>
-      <c r="C106" s="2"/>
+      <c r="A106" s="5"/>
+      <c r="B106" s="5"/>
+      <c r="C106" s="5"/>
       <c r="D106" s="3" t="s">
         <v>134</v>
       </c>
       <c r="E106" s="3"/>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A107" s="2"/>
-      <c r="B107" s="2"/>
-      <c r="C107" s="2"/>
+      <c r="A107" s="5"/>
+      <c r="B107" s="5"/>
+      <c r="C107" s="5"/>
       <c r="D107" s="3" t="s">
         <v>135</v>
       </c>
       <c r="E107" s="3"/>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A108" s="2"/>
-      <c r="B108" s="2"/>
-      <c r="C108" s="2"/>
+      <c r="A108" s="5"/>
+      <c r="B108" s="5"/>
+      <c r="C108" s="5"/>
       <c r="D108" s="3" t="s">
         <v>130</v>
       </c>
       <c r="E108" s="3"/>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A109" s="2"/>
-      <c r="B109" s="2"/>
-      <c r="C109" s="2" t="s">
+      <c r="A109" s="5"/>
+      <c r="B109" s="5"/>
+      <c r="C109" s="5" t="s">
         <v>136</v>
       </c>
       <c r="D109" s="3" t="s">
@@ -2054,36 +2177,36 @@
       <c r="E109" s="3"/>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A110" s="2"/>
-      <c r="B110" s="2"/>
-      <c r="C110" s="2"/>
+      <c r="A110" s="5"/>
+      <c r="B110" s="5"/>
+      <c r="C110" s="5"/>
       <c r="D110" s="3" t="s">
         <v>138</v>
       </c>
       <c r="E110" s="3"/>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A111" s="2"/>
-      <c r="B111" s="2"/>
-      <c r="C111" s="2"/>
+      <c r="A111" s="5"/>
+      <c r="B111" s="5"/>
+      <c r="C111" s="5"/>
       <c r="D111" s="3" t="s">
         <v>139</v>
       </c>
       <c r="E111" s="3"/>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A112" s="2"/>
-      <c r="B112" s="2"/>
-      <c r="C112" s="2"/>
+      <c r="A112" s="5"/>
+      <c r="B112" s="5"/>
+      <c r="C112" s="5"/>
       <c r="D112" s="3" t="s">
         <v>140</v>
       </c>
       <c r="E112" s="3"/>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A113" s="2"/>
-      <c r="B113" s="2"/>
-      <c r="C113" s="2" t="s">
+      <c r="A113" s="5"/>
+      <c r="B113" s="5"/>
+      <c r="C113" s="5" t="s">
         <v>141</v>
       </c>
       <c r="D113" s="3" t="s">
@@ -2092,31 +2215,31 @@
       <c r="E113" s="3"/>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A114" s="2"/>
-      <c r="B114" s="2"/>
-      <c r="C114" s="2"/>
+      <c r="A114" s="5"/>
+      <c r="B114" s="5"/>
+      <c r="C114" s="5"/>
       <c r="D114" s="3" t="s">
         <v>143</v>
       </c>
       <c r="E114" s="3"/>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A115" s="2"/>
-      <c r="B115" s="2"/>
-      <c r="C115" s="2"/>
+      <c r="A115" s="5"/>
+      <c r="B115" s="5"/>
+      <c r="C115" s="5"/>
       <c r="D115" s="3" t="s">
         <v>144</v>
       </c>
       <c r="E115" s="3"/>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A116" s="2" t="s">
+      <c r="A116" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="B116" s="2" t="s">
+      <c r="B116" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="C116" s="2" t="s">
+      <c r="C116" s="5" t="s">
         <v>147</v>
       </c>
       <c r="D116" s="3" t="s">
@@ -2125,45 +2248,45 @@
       <c r="E116" s="3"/>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A117" s="2"/>
-      <c r="B117" s="2"/>
-      <c r="C117" s="2"/>
+      <c r="A117" s="5"/>
+      <c r="B117" s="5"/>
+      <c r="C117" s="5"/>
       <c r="D117" s="3" t="s">
         <v>149</v>
       </c>
       <c r="E117" s="3"/>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A118" s="2"/>
-      <c r="B118" s="2"/>
-      <c r="C118" s="2"/>
+      <c r="A118" s="5"/>
+      <c r="B118" s="5"/>
+      <c r="C118" s="5"/>
       <c r="D118" s="3" t="s">
         <v>150</v>
       </c>
       <c r="E118" s="3"/>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A119" s="2"/>
-      <c r="B119" s="2"/>
-      <c r="C119" s="2"/>
+      <c r="A119" s="5"/>
+      <c r="B119" s="5"/>
+      <c r="C119" s="5"/>
       <c r="D119" s="3" t="s">
         <v>151</v>
       </c>
       <c r="E119" s="3"/>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A120" s="2"/>
-      <c r="B120" s="2"/>
-      <c r="C120" s="2"/>
+      <c r="A120" s="5"/>
+      <c r="B120" s="5"/>
+      <c r="C120" s="5"/>
       <c r="D120" s="3" t="s">
         <v>152</v>
       </c>
       <c r="E120" s="3"/>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A121" s="2"/>
-      <c r="B121" s="2"/>
-      <c r="C121" s="2" t="s">
+      <c r="A121" s="5"/>
+      <c r="B121" s="5"/>
+      <c r="C121" s="5" t="s">
         <v>153</v>
       </c>
       <c r="D121" s="3" t="s">
@@ -2172,45 +2295,45 @@
       <c r="E121" s="3"/>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A122" s="2"/>
-      <c r="B122" s="2"/>
-      <c r="C122" s="2"/>
+      <c r="A122" s="5"/>
+      <c r="B122" s="5"/>
+      <c r="C122" s="5"/>
       <c r="D122" s="3" t="s">
         <v>155</v>
       </c>
       <c r="E122" s="3"/>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A123" s="2"/>
-      <c r="B123" s="2"/>
-      <c r="C123" s="2"/>
+      <c r="A123" s="5"/>
+      <c r="B123" s="5"/>
+      <c r="C123" s="5"/>
       <c r="D123" s="3" t="s">
         <v>156</v>
       </c>
       <c r="E123" s="3"/>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A124" s="2"/>
-      <c r="B124" s="2"/>
-      <c r="C124" s="2"/>
+      <c r="A124" s="5"/>
+      <c r="B124" s="5"/>
+      <c r="C124" s="5"/>
       <c r="D124" s="3" t="s">
         <v>157</v>
       </c>
       <c r="E124" s="3"/>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A125" s="2"/>
-      <c r="B125" s="2"/>
-      <c r="C125" s="2"/>
+      <c r="A125" s="5"/>
+      <c r="B125" s="5"/>
+      <c r="C125" s="5"/>
       <c r="D125" s="3" t="s">
         <v>158</v>
       </c>
       <c r="E125" s="3"/>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A126" s="2"/>
-      <c r="B126" s="2"/>
-      <c r="C126" s="2" t="s">
+      <c r="A126" s="5"/>
+      <c r="B126" s="5"/>
+      <c r="C126" s="5" t="s">
         <v>159</v>
       </c>
       <c r="D126" s="3" t="s">
@@ -2219,94 +2342,94 @@
       <c r="E126" s="3"/>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A127" s="2"/>
-      <c r="B127" s="2"/>
-      <c r="C127" s="2"/>
+      <c r="A127" s="5"/>
+      <c r="B127" s="5"/>
+      <c r="C127" s="5"/>
       <c r="D127" s="3" t="s">
         <v>160</v>
       </c>
       <c r="E127" s="3"/>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A128" s="2"/>
-      <c r="B128" s="2"/>
-      <c r="C128" s="2"/>
+      <c r="A128" s="5"/>
+      <c r="B128" s="5"/>
+      <c r="C128" s="5"/>
       <c r="D128" s="3" t="s">
         <v>26</v>
       </c>
       <c r="E128" s="3"/>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A129" s="2"/>
-      <c r="B129" s="2"/>
-      <c r="C129" s="2"/>
+      <c r="A129" s="5"/>
+      <c r="B129" s="5"/>
+      <c r="C129" s="5"/>
       <c r="D129" s="3" t="s">
         <v>21</v>
       </c>
       <c r="E129" s="3"/>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A130" s="2"/>
-      <c r="B130" s="2"/>
-      <c r="C130" s="2"/>
+      <c r="A130" s="5"/>
+      <c r="B130" s="5"/>
+      <c r="C130" s="5"/>
       <c r="D130" s="3" t="s">
         <v>28</v>
       </c>
       <c r="E130" s="3"/>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A131" s="2"/>
-      <c r="B131" s="2"/>
-      <c r="C131" s="2"/>
+      <c r="A131" s="5"/>
+      <c r="B131" s="5"/>
+      <c r="C131" s="5"/>
       <c r="D131" s="3" t="s">
         <v>25</v>
       </c>
       <c r="E131" s="3"/>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A132" s="2"/>
-      <c r="B132" s="2"/>
-      <c r="C132" s="2"/>
+      <c r="A132" s="5"/>
+      <c r="B132" s="5"/>
+      <c r="C132" s="5"/>
       <c r="D132" s="3" t="s">
         <v>161</v>
       </c>
       <c r="E132" s="3"/>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A133" s="2"/>
-      <c r="B133" s="2"/>
-      <c r="C133" s="2"/>
+      <c r="A133" s="5"/>
+      <c r="B133" s="5"/>
+      <c r="C133" s="5"/>
       <c r="D133" s="3" t="s">
         <v>162</v>
       </c>
       <c r="E133" s="3"/>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A134" s="2"/>
-      <c r="B134" s="2"/>
-      <c r="C134" s="2"/>
+      <c r="A134" s="5"/>
+      <c r="B134" s="5"/>
+      <c r="C134" s="5"/>
       <c r="D134" s="3" t="s">
         <v>30</v>
       </c>
       <c r="E134" s="3"/>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A135" s="2"/>
-      <c r="B135" s="2"/>
-      <c r="C135" s="2"/>
+      <c r="A135" s="5"/>
+      <c r="B135" s="5"/>
+      <c r="C135" s="5"/>
       <c r="D135" s="3" t="s">
         <v>29</v>
       </c>
       <c r="E135" s="3"/>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A136" s="2" t="s">
+      <c r="A136" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="B136" s="2" t="s">
+      <c r="B136" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="C136" s="2" t="s">
+      <c r="C136" s="5" t="s">
         <v>165</v>
       </c>
       <c r="D136" s="3" t="s">
@@ -2315,27 +2438,27 @@
       <c r="E136" s="3"/>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A137" s="2"/>
-      <c r="B137" s="2"/>
-      <c r="C137" s="2"/>
+      <c r="A137" s="5"/>
+      <c r="B137" s="5"/>
+      <c r="C137" s="5"/>
       <c r="D137" s="3" t="s">
         <v>167</v>
       </c>
       <c r="E137" s="3"/>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A138" s="2"/>
-      <c r="B138" s="2"/>
-      <c r="C138" s="2"/>
+      <c r="A138" s="5"/>
+      <c r="B138" s="5"/>
+      <c r="C138" s="5"/>
       <c r="D138" s="3" t="s">
         <v>168</v>
       </c>
       <c r="E138" s="3"/>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A139" s="2"/>
-      <c r="B139" s="2"/>
-      <c r="C139" s="2" t="s">
+      <c r="A139" s="5"/>
+      <c r="B139" s="5"/>
+      <c r="C139" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D139" s="3" t="s">
@@ -2344,27 +2467,27 @@
       <c r="E139" s="3"/>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A140" s="2"/>
-      <c r="B140" s="2"/>
-      <c r="C140" s="2"/>
+      <c r="A140" s="5"/>
+      <c r="B140" s="5"/>
+      <c r="C140" s="5"/>
       <c r="D140" s="3" t="s">
         <v>170</v>
       </c>
       <c r="E140" s="3"/>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A141" s="2"/>
-      <c r="B141" s="2"/>
-      <c r="C141" s="2"/>
+      <c r="A141" s="5"/>
+      <c r="B141" s="5"/>
+      <c r="C141" s="5"/>
       <c r="D141" s="3" t="s">
         <v>171</v>
       </c>
       <c r="E141" s="3"/>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A142" s="2"/>
-      <c r="B142" s="2"/>
-      <c r="C142" s="2" t="s">
+      <c r="A142" s="5"/>
+      <c r="B142" s="5"/>
+      <c r="C142" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D142" s="3" t="s">
@@ -2373,36 +2496,36 @@
       <c r="E142" s="3"/>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A143" s="2"/>
-      <c r="B143" s="2"/>
-      <c r="C143" s="2"/>
+      <c r="A143" s="5"/>
+      <c r="B143" s="5"/>
+      <c r="C143" s="5"/>
       <c r="D143" s="3" t="s">
         <v>180</v>
       </c>
       <c r="E143" s="3"/>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A144" s="2"/>
-      <c r="B144" s="2"/>
-      <c r="C144" s="2"/>
+      <c r="A144" s="5"/>
+      <c r="B144" s="5"/>
+      <c r="C144" s="5"/>
       <c r="D144" s="3" t="s">
         <v>181</v>
       </c>
       <c r="E144" s="3"/>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A145" s="2"/>
-      <c r="B145" s="2"/>
-      <c r="C145" s="2"/>
+      <c r="A145" s="5"/>
+      <c r="B145" s="5"/>
+      <c r="C145" s="5"/>
       <c r="D145" s="3" t="s">
         <v>182</v>
       </c>
       <c r="E145" s="3"/>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A146" s="2"/>
-      <c r="B146" s="2"/>
-      <c r="C146" s="2" t="s">
+      <c r="A146" s="5"/>
+      <c r="B146" s="5"/>
+      <c r="C146" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D146" s="3" t="s">
@@ -2411,18 +2534,18 @@
       <c r="E146" s="3"/>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A147" s="2"/>
-      <c r="B147" s="2"/>
-      <c r="C147" s="2"/>
+      <c r="A147" s="5"/>
+      <c r="B147" s="5"/>
+      <c r="C147" s="5"/>
       <c r="D147" s="3" t="s">
         <v>173</v>
       </c>
       <c r="E147" s="3"/>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A148" s="2"/>
-      <c r="B148" s="2"/>
-      <c r="C148" s="2" t="s">
+      <c r="A148" s="5"/>
+      <c r="B148" s="5"/>
+      <c r="C148" s="5" t="s">
         <v>174</v>
       </c>
       <c r="D148" s="3" t="s">
@@ -2431,27 +2554,166 @@
       <c r="E148" s="3"/>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A149" s="2"/>
-      <c r="B149" s="2"/>
-      <c r="C149" s="2"/>
+      <c r="A149" s="5"/>
+      <c r="B149" s="5"/>
+      <c r="C149" s="5"/>
       <c r="D149" s="3" t="s">
         <v>176</v>
       </c>
       <c r="E149" s="3"/>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A150" s="2"/>
-      <c r="B150" s="2"/>
-      <c r="C150" s="1" t="s">
+      <c r="A150" s="7"/>
+      <c r="B150" s="7"/>
+      <c r="C150" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="D150" s="3" t="s">
+      <c r="D150" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="E150" s="3"/>
+      <c r="E150" s="9"/>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A151" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="B151" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="C151" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="D151" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="E151" s="3"/>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A152" s="5"/>
+      <c r="B152" s="5"/>
+      <c r="C152" s="5"/>
+      <c r="D152" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="E152" s="3"/>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A153" s="5"/>
+      <c r="B153" s="5"/>
+      <c r="C153" s="5"/>
+      <c r="D153" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="E153" s="3"/>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A154" s="5"/>
+      <c r="B154" s="5"/>
+      <c r="C154" s="5"/>
+      <c r="D154" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="E154" s="3"/>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A155" s="5"/>
+      <c r="B155" s="5"/>
+      <c r="C155" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="D155" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="E155" s="3"/>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A156" s="5"/>
+      <c r="B156" s="5"/>
+      <c r="C156" s="5"/>
+      <c r="D156" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="E156" s="3"/>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A157" s="5"/>
+      <c r="B157" s="5"/>
+      <c r="C157" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="D157" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="E157" s="3"/>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A158" s="5"/>
+      <c r="B158" s="5"/>
+      <c r="C158" s="5"/>
+      <c r="D158" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E158" s="3"/>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A159" s="5"/>
+      <c r="B159" s="5"/>
+      <c r="C159" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="D159" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="E159" s="3"/>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A160" s="5"/>
+      <c r="B160" s="5"/>
+      <c r="C160" s="5"/>
+      <c r="D160" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="E160" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="40">
+  <mergeCells count="48">
+    <mergeCell ref="A151:A160"/>
+    <mergeCell ref="H1:H4"/>
+    <mergeCell ref="H5:H7"/>
+    <mergeCell ref="C151:C154"/>
+    <mergeCell ref="C155:C156"/>
+    <mergeCell ref="C157:C158"/>
+    <mergeCell ref="C159:C160"/>
+    <mergeCell ref="B151:B160"/>
+    <mergeCell ref="C60:C71"/>
+    <mergeCell ref="A2:A12"/>
+    <mergeCell ref="B2:B12"/>
+    <mergeCell ref="B13:B32"/>
+    <mergeCell ref="A13:A32"/>
+    <mergeCell ref="B33:B37"/>
+    <mergeCell ref="A33:A37"/>
+    <mergeCell ref="C24:C32"/>
+    <mergeCell ref="C13:C23"/>
+    <mergeCell ref="C38:C49"/>
+    <mergeCell ref="C50:C52"/>
+    <mergeCell ref="C53:C59"/>
+    <mergeCell ref="B38:B71"/>
+    <mergeCell ref="A38:A71"/>
+    <mergeCell ref="B72:B81"/>
+    <mergeCell ref="A72:A81"/>
+    <mergeCell ref="B82:B86"/>
+    <mergeCell ref="A82:A86"/>
+    <mergeCell ref="C87:C91"/>
+    <mergeCell ref="C94:C98"/>
+    <mergeCell ref="B87:B98"/>
+    <mergeCell ref="A87:A98"/>
+    <mergeCell ref="C99:C103"/>
+    <mergeCell ref="C109:C112"/>
+    <mergeCell ref="C113:C115"/>
+    <mergeCell ref="B99:B115"/>
+    <mergeCell ref="A99:A115"/>
+    <mergeCell ref="C116:C120"/>
+    <mergeCell ref="C104:C108"/>
     <mergeCell ref="C146:C147"/>
     <mergeCell ref="C148:C149"/>
     <mergeCell ref="B136:B150"/>
@@ -2462,36 +2724,7 @@
     <mergeCell ref="C136:C138"/>
     <mergeCell ref="C139:C141"/>
     <mergeCell ref="C142:C145"/>
-    <mergeCell ref="C109:C112"/>
-    <mergeCell ref="C113:C115"/>
-    <mergeCell ref="B99:B115"/>
-    <mergeCell ref="A99:A115"/>
-    <mergeCell ref="C116:C120"/>
     <mergeCell ref="C121:C125"/>
-    <mergeCell ref="C87:C91"/>
-    <mergeCell ref="C94:C98"/>
-    <mergeCell ref="B87:B98"/>
-    <mergeCell ref="A87:A98"/>
-    <mergeCell ref="C99:C103"/>
-    <mergeCell ref="C104:C108"/>
-    <mergeCell ref="B38:B71"/>
-    <mergeCell ref="A38:A71"/>
-    <mergeCell ref="B72:B81"/>
-    <mergeCell ref="A72:A81"/>
-    <mergeCell ref="B82:B86"/>
-    <mergeCell ref="A82:A86"/>
-    <mergeCell ref="C24:C32"/>
-    <mergeCell ref="C13:C23"/>
-    <mergeCell ref="C38:C49"/>
-    <mergeCell ref="C50:C52"/>
-    <mergeCell ref="C53:C59"/>
-    <mergeCell ref="C60:C71"/>
-    <mergeCell ref="A2:A12"/>
-    <mergeCell ref="B2:B12"/>
-    <mergeCell ref="B13:B32"/>
-    <mergeCell ref="A13:A32"/>
-    <mergeCell ref="B33:B37"/>
-    <mergeCell ref="A33:A37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>